<commit_message>
ajustes de vista de eventos
</commit_message>
<xml_diff>
--- a/lista_eventos_vl550v4.xlsx
+++ b/lista_eventos_vl550v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{432BDAF2-7904-42B2-B3A8-D8B4E1EFAF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{432BDAF2-7904-42B2-B3A8-D8B4E1EFAF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59373BE3-AEA4-424B-BC9A-7F82527FA69A}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="117">
   <si>
     <t>ID</t>
   </si>
@@ -381,6 +381,15 @@
   </si>
   <si>
     <t>latitude</t>
+  </si>
+  <si>
+    <t>[*/*/*-*:*:*.*][UpdateHandler][T]Update requested!!!
+[*/*/*-*:*:*.*][UpdateHandler][T]State: EXECUTE_UPDATE
+[*/*/*-*:*:*.*][UpdateHandler][T]UpdateState: UPDATE_NOW
+[*/*/*-*:*:*.*][UpdateHandler][T]Ready to update!</t>
+  </si>
+  <si>
+    <t>actualizacion de FW en curso!</t>
   </si>
 </sst>
 </file>
@@ -404,7 +413,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -521,17 +530,6 @@
       <right style="thick">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -597,11 +595,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1477,10 +1477,10 @@
       <c r="B49" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="C49" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="D49" s="17"/>
+      <c r="D49" s="16"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
@@ -1489,10 +1489,10 @@
       <c r="B50" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="C50" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D50" s="17"/>
+      <c r="D50" s="16"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
@@ -1501,10 +1501,10 @@
       <c r="B51" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="C51" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D51" s="17"/>
+      <c r="D51" s="16"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="7">
@@ -1513,10 +1513,10 @@
       <c r="B52" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="C52" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D52" s="17"/>
+      <c r="D52" s="16"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="7">
@@ -1525,100 +1525,106 @@
       <c r="B53" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C53" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D53" s="17"/>
+      <c r="D53" s="16"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" s="12">
+      <c r="A54" s="7">
         <v>53</v>
       </c>
       <c r="B54" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C54" s="15" t="s">
+      <c r="C54" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D54" s="17"/>
+      <c r="D54" s="16"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" s="12">
+      <c r="A55" s="7">
         <v>54</v>
       </c>
       <c r="B55" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C55" s="15" t="s">
+      <c r="C55" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D55" s="17"/>
+      <c r="D55" s="16"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="12">
+      <c r="A56" s="7">
         <v>55</v>
       </c>
       <c r="B56" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="15" t="s">
+      <c r="C56" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D56" s="17"/>
+      <c r="D56" s="16"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="12">
-        <v>55</v>
+      <c r="A57" s="7">
+        <v>56</v>
       </c>
       <c r="B57" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="15" t="s">
+      <c r="C57" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D57" s="17"/>
+      <c r="D57" s="16"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="12">
-        <v>55</v>
+      <c r="A58" s="7">
+        <v>57</v>
       </c>
       <c r="B58" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C58" s="15" t="s">
+      <c r="C58" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D58" s="17"/>
+      <c r="D58" s="16"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="13">
-        <v>55</v>
-      </c>
-      <c r="B59" s="14" t="s">
+      <c r="A59" s="7">
+        <v>58</v>
+      </c>
+      <c r="B59" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C59" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D59" s="17"/>
+      <c r="D59" s="16"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="13">
-        <v>55</v>
-      </c>
-      <c r="B60" s="14" t="s">
+      <c r="A60" s="7">
+        <v>59</v>
+      </c>
+      <c r="B60" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D60" s="17"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="13"/>
-      <c r="B61" s="8"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="17"/>
+      <c r="D60" s="16"/>
+    </row>
+    <row r="61" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="A61" s="12">
+        <v>60</v>
+      </c>
+      <c r="B61" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C61" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D61" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>